<commit_message>
Subiendo imagenes de cambios enero 2026
</commit_message>
<xml_diff>
--- a/storage/app/pdfs/ghg_asia_download.xlsx
+++ b/storage/app/pdfs/ghg_asia_download.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rodrigofavela/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rodrigofavela/Desktop/Cambio EthTool/Vietnam/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D959BECF-24C2-5B44-8479-9BCE34316C50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502085D9-ECB0-4148-96CB-83DF2292C891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5520" yWindow="4140" windowWidth="23280" windowHeight="12480" tabRatio="853" xr2:uid="{AD60D5F5-4EC3-4F16-A51A-8F435208B142}"/>
+    <workbookView xWindow="5520" yWindow="4140" windowWidth="23280" windowHeight="12480" tabRatio="853" activeTab="6" xr2:uid="{AD60D5F5-4EC3-4F16-A51A-8F435208B142}"/>
   </bookViews>
   <sheets>
     <sheet name="Content" sheetId="7" r:id="rId1"/>
@@ -10097,7 +10097,7 @@
   <sheetPr>
     <tabColor rgb="FFD18316"/>
   </sheetPr>
-  <dimension ref="A1:W111"/>
+  <dimension ref="A1:W101"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="27" style="8" bestFit="1" customWidth="1"/>
@@ -10138,7 +10138,7 @@
       <c r="M4" s="17"/>
       <c r="N4" s="17"/>
     </row>
-    <row r="5" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="18" t="s">
         <v>10</v>
       </c>
@@ -10169,8 +10169,15 @@
       <c r="L5" s="17"/>
       <c r="M5" s="17"/>
       <c r="N5" s="17"/>
-    </row>
-    <row r="6" spans="1:23" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="Q5" s="12"/>
+      <c r="R5" s="12"/>
+      <c r="S5" s="12"/>
+      <c r="T5" s="12"/>
+      <c r="U5" s="12"/>
+      <c r="V5" s="12"/>
+      <c r="W5" s="12"/>
+    </row>
+    <row r="6" spans="1:23" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="21" t="s">
         <v>18</v>
       </c>
@@ -10178,22 +10185,22 @@
         <v>19</v>
       </c>
       <c r="C6" s="23">
-        <v>48.283108136252032</v>
+        <v>48.949325901782046</v>
       </c>
       <c r="D6" s="23">
-        <v>41.909095364152577</v>
+        <v>42.459046339124036</v>
       </c>
       <c r="E6" s="23">
-        <v>40.344893885623236</v>
+        <v>40.833629488308716</v>
       </c>
       <c r="F6" s="23">
-        <v>39.085918227964541</v>
+        <v>39.511235956118341</v>
       </c>
       <c r="G6" s="23">
-        <v>37.919988167232162</v>
+        <v>38.279564473435236</v>
       </c>
       <c r="H6" s="23">
-        <v>36.319930400557901</v>
+        <v>36.61131165682395</v>
       </c>
       <c r="I6" s="17"/>
       <c r="J6" s="17"/>
@@ -10209,7 +10216,7 @@
       <c r="V6" s="12"/>
       <c r="W6" s="12"/>
     </row>
-    <row r="7" spans="1:23" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:23" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="21" t="s">
         <v>20</v>
       </c>
@@ -10217,22 +10224,22 @@
         <v>19</v>
       </c>
       <c r="C7" s="23">
-        <v>71.368566639406922</v>
+        <v>75.026221645356188</v>
       </c>
       <c r="D7" s="23">
-        <v>64.381372523284568</v>
+        <v>67.84330407519208</v>
       </c>
       <c r="E7" s="23">
-        <v>62.534364542885932</v>
+        <v>65.898434367772566</v>
       </c>
       <c r="F7" s="23">
-        <v>61.009579488799346</v>
+        <v>64.275787586665103</v>
       </c>
       <c r="G7" s="23">
-        <v>59.595771264424748</v>
+        <v>62.764117635269635</v>
       </c>
       <c r="H7" s="23">
-        <v>57.766770421996732</v>
+        <v>60.837255065820749</v>
       </c>
       <c r="I7" s="17"/>
       <c r="J7" s="17"/>
@@ -10248,7 +10255,7 @@
       <c r="V7" s="12"/>
       <c r="W7" s="12"/>
     </row>
-    <row r="8" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A8" s="18" t="s">
         <v>21</v>
       </c>
@@ -10287,7 +10294,7 @@
       <c r="V8" s="12"/>
       <c r="W8" s="12"/>
     </row>
-    <row r="9" spans="1:23" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:23" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
         <v>18</v>
       </c>
@@ -10298,19 +10305,19 @@
         <v>0</v>
       </c>
       <c r="D9" s="25">
-        <v>0.13201330689218213</v>
+        <v>0.13259180679384444</v>
       </c>
       <c r="E9" s="25">
-        <v>0.16440976061913065</v>
+        <v>0.16579791986834838</v>
       </c>
       <c r="F9" s="25">
-        <v>0.19048462833696567</v>
+        <v>0.19281348152988767</v>
       </c>
       <c r="G9" s="25">
-        <v>0.21463241222532251</v>
+        <v>0.21797565608474226</v>
       </c>
       <c r="H9" s="26">
-        <v>0.24777149188355402</v>
+        <v>0.25205687754954187</v>
       </c>
       <c r="I9" s="17"/>
       <c r="J9" s="17"/>
@@ -10326,7 +10333,7 @@
       <c r="V9" s="12"/>
       <c r="W9" s="12"/>
     </row>
-    <row r="10" spans="1:23" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:23" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="21" t="s">
         <v>20</v>
       </c>
@@ -10337,19 +10344,19 @@
         <v>0</v>
       </c>
       <c r="D10" s="25">
-        <v>9.7902962678590472E-2</v>
+        <v>9.5738761897370586E-2</v>
       </c>
       <c r="E10" s="25">
-        <v>0.12378281521550259</v>
+        <v>0.12166129491006554</v>
       </c>
       <c r="F10" s="25">
-        <v>0.1451477539537378</v>
+        <v>0.14328902379634217</v>
       </c>
       <c r="G10" s="25">
-        <v>0.16495771078694604</v>
+        <v>0.1634375787714418</v>
       </c>
       <c r="H10" s="26">
-        <v>0.19058525143336438</v>
+        <v>0.18912010052439682</v>
       </c>
       <c r="I10" s="17"/>
       <c r="J10" s="17"/>
@@ -10365,7 +10372,7 @@
       <c r="V10" s="12"/>
       <c r="W10" s="12"/>
     </row>
-    <row r="11" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A11" s="18" t="s">
         <v>23</v>
       </c>
@@ -10404,7 +10411,7 @@
       <c r="V11" s="12"/>
       <c r="W11" s="12"/>
     </row>
-    <row r="12" spans="1:23" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:23" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="21" t="s">
         <v>18</v>
       </c>
@@ -10415,19 +10422,19 @@
         <v>0</v>
       </c>
       <c r="D12" s="25">
-        <v>4.0001278623531845E-2</v>
+        <v>4.07309320538096E-2</v>
       </c>
       <c r="E12" s="25">
-        <v>4.9817710030741515E-2</v>
+        <v>5.0931531684461358E-2</v>
       </c>
       <c r="F12" s="25">
-        <v>5.7718641180846825E-2</v>
+        <v>5.9230453262191493E-2</v>
       </c>
       <c r="G12" s="25">
-        <v>6.5035647732678004E-2</v>
+        <v>6.6960032086872373E-2</v>
       </c>
       <c r="H12" s="26">
-        <v>7.5077101809871774E-2</v>
+        <v>7.7429456626443821E-2</v>
       </c>
       <c r="I12" s="17"/>
       <c r="J12" s="17"/>
@@ -10443,7 +10450,7 @@
       <c r="V12" s="12"/>
       <c r="W12" s="12"/>
     </row>
-    <row r="13" spans="1:23" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:23" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="21" t="s">
         <v>20</v>
       </c>
@@ -10454,19 +10461,19 @@
         <v>0</v>
       </c>
       <c r="D13" s="27">
-        <v>4.3849409881814953E-2</v>
+        <v>4.5077708082369938E-2</v>
       </c>
       <c r="E13" s="27">
-        <v>5.5440645024489046E-2</v>
+        <v>5.728309232532152E-2</v>
       </c>
       <c r="F13" s="27">
-        <v>6.5009711477649723E-2</v>
+        <v>6.7466307878759693E-2</v>
       </c>
       <c r="G13" s="27">
-        <v>7.3882322613761625E-2</v>
+        <v>7.6953068115149043E-2</v>
       </c>
       <c r="H13" s="28">
-        <v>8.5360550680841502E-2</v>
+        <v>8.9045445282506366E-2</v>
       </c>
       <c r="I13" s="17"/>
       <c r="J13" s="17"/>
@@ -10482,7 +10489,7 @@
       <c r="V13" s="12"/>
       <c r="W13" s="12"/>
     </row>
-    <row r="14" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A14" s="17"/>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
@@ -10497,15 +10504,15 @@
       <c r="L14" s="17"/>
       <c r="M14" s="17"/>
       <c r="N14" s="17"/>
-      <c r="Q14" s="12"/>
-      <c r="R14" s="12"/>
-      <c r="S14" s="12"/>
-      <c r="T14" s="12"/>
-      <c r="U14" s="12"/>
-      <c r="V14" s="12"/>
-      <c r="W14" s="12"/>
-    </row>
-    <row r="15" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="Q14" s="16"/>
+      <c r="R14" s="13"/>
+      <c r="S14" s="13"/>
+      <c r="T14" s="13"/>
+      <c r="U14" s="13"/>
+      <c r="V14" s="13"/>
+      <c r="W14" s="13"/>
+    </row>
+    <row r="15" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="17"/>
       <c r="B15" s="17"/>
       <c r="C15" s="17"/>
@@ -10520,13 +10527,13 @@
       <c r="L15" s="17"/>
       <c r="M15" s="17"/>
       <c r="N15" s="17"/>
-      <c r="Q15" s="12"/>
-      <c r="R15" s="12"/>
-      <c r="S15" s="12"/>
-      <c r="T15" s="12"/>
-      <c r="U15" s="12"/>
-      <c r="V15" s="12"/>
-      <c r="W15" s="12"/>
+      <c r="Q15" s="15"/>
+      <c r="R15" s="14"/>
+      <c r="S15" s="14"/>
+      <c r="T15" s="14"/>
+      <c r="U15" s="14"/>
+      <c r="V15" s="14"/>
+      <c r="W15" s="14"/>
     </row>
     <row r="16" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="17"/>
@@ -10543,15 +10550,8 @@
       <c r="L16" s="17"/>
       <c r="M16" s="17"/>
       <c r="N16" s="17"/>
-      <c r="Q16" s="12"/>
-      <c r="R16" s="12"/>
-      <c r="S16" s="12"/>
-      <c r="T16" s="12"/>
-      <c r="U16" s="12"/>
-      <c r="V16" s="12"/>
-      <c r="W16" s="12"/>
-    </row>
-    <row r="17" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="17"/>
       <c r="B17" s="17"/>
       <c r="C17" s="17"/>
@@ -10566,15 +10566,8 @@
       <c r="L17" s="17"/>
       <c r="M17" s="17"/>
       <c r="N17" s="17"/>
-      <c r="Q17" s="12"/>
-      <c r="R17" s="12"/>
-      <c r="S17" s="12"/>
-      <c r="T17" s="12"/>
-      <c r="U17" s="12"/>
-      <c r="V17" s="12"/>
-      <c r="W17" s="12"/>
-    </row>
-    <row r="18" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:22" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="17"/>
       <c r="B18" s="17"/>
       <c r="C18" s="17"/>
@@ -10589,15 +10582,8 @@
       <c r="L18" s="17"/>
       <c r="M18" s="17"/>
       <c r="N18" s="17"/>
-      <c r="Q18" s="12"/>
-      <c r="R18" s="12"/>
-      <c r="S18" s="12"/>
-      <c r="T18" s="12"/>
-      <c r="U18" s="12"/>
-      <c r="V18" s="12"/>
-      <c r="W18" s="12"/>
-    </row>
-    <row r="19" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="17"/>
       <c r="B19" s="17"/>
       <c r="C19" s="17"/>
@@ -10612,15 +10598,8 @@
       <c r="L19" s="17"/>
       <c r="M19" s="17"/>
       <c r="N19" s="17"/>
-      <c r="Q19" s="12"/>
-      <c r="R19" s="12"/>
-      <c r="S19" s="12"/>
-      <c r="T19" s="12"/>
-      <c r="U19" s="12"/>
-      <c r="V19" s="12"/>
-      <c r="W19" s="12"/>
-    </row>
-    <row r="20" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A20" s="17"/>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
@@ -10635,15 +10614,9 @@
       <c r="L20" s="17"/>
       <c r="M20" s="17"/>
       <c r="N20" s="17"/>
-      <c r="Q20" s="12"/>
-      <c r="R20" s="12"/>
-      <c r="S20" s="12"/>
-      <c r="T20" s="12"/>
-      <c r="U20" s="12"/>
-      <c r="V20" s="12"/>
-      <c r="W20" s="12"/>
-    </row>
-    <row r="21" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="O20" s="9"/>
+    </row>
+    <row r="21" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A21" s="17"/>
       <c r="B21" s="17"/>
       <c r="C21" s="17"/>
@@ -10658,15 +10631,15 @@
       <c r="L21" s="17"/>
       <c r="M21" s="17"/>
       <c r="N21" s="17"/>
+      <c r="O21" s="9"/>
       <c r="Q21" s="12"/>
       <c r="R21" s="12"/>
       <c r="S21" s="12"/>
       <c r="T21" s="12"/>
       <c r="U21" s="12"/>
       <c r="V21" s="12"/>
-      <c r="W21" s="12"/>
-    </row>
-    <row r="22" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A22" s="17"/>
       <c r="B22" s="17"/>
       <c r="C22" s="17"/>
@@ -10681,15 +10654,15 @@
       <c r="L22" s="17"/>
       <c r="M22" s="17"/>
       <c r="N22" s="17"/>
+      <c r="O22" s="9"/>
       <c r="Q22" s="12"/>
       <c r="R22" s="12"/>
       <c r="S22" s="12"/>
       <c r="T22" s="12"/>
       <c r="U22" s="12"/>
       <c r="V22" s="12"/>
-      <c r="W22" s="12"/>
-    </row>
-    <row r="23" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A23" s="17"/>
       <c r="B23" s="17"/>
       <c r="C23" s="17"/>
@@ -10704,15 +10677,15 @@
       <c r="L23" s="17"/>
       <c r="M23" s="17"/>
       <c r="N23" s="17"/>
+      <c r="O23" s="9"/>
       <c r="Q23" s="12"/>
       <c r="R23" s="12"/>
       <c r="S23" s="12"/>
       <c r="T23" s="12"/>
       <c r="U23" s="12"/>
       <c r="V23" s="12"/>
-      <c r="W23" s="12"/>
-    </row>
-    <row r="24" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A24" s="17"/>
       <c r="B24" s="17"/>
       <c r="C24" s="17"/>
@@ -10727,15 +10700,15 @@
       <c r="L24" s="17"/>
       <c r="M24" s="17"/>
       <c r="N24" s="17"/>
-      <c r="Q24" s="16"/>
-      <c r="R24" s="13"/>
-      <c r="S24" s="13"/>
-      <c r="T24" s="13"/>
-      <c r="U24" s="13"/>
-      <c r="V24" s="13"/>
-      <c r="W24" s="13"/>
-    </row>
-    <row r="25" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="O24" s="9"/>
+      <c r="Q24" s="12"/>
+      <c r="R24" s="12"/>
+      <c r="S24" s="12"/>
+      <c r="T24" s="12"/>
+      <c r="U24" s="12"/>
+      <c r="V24" s="12"/>
+    </row>
+    <row r="25" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A25" s="17"/>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
@@ -10750,15 +10723,15 @@
       <c r="L25" s="17"/>
       <c r="M25" s="17"/>
       <c r="N25" s="17"/>
-      <c r="Q25" s="15"/>
-      <c r="R25" s="14"/>
-      <c r="S25" s="14"/>
-      <c r="T25" s="14"/>
-      <c r="U25" s="14"/>
-      <c r="V25" s="14"/>
-      <c r="W25" s="14"/>
-    </row>
-    <row r="26" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="O25" s="9"/>
+      <c r="Q25" s="12"/>
+      <c r="R25" s="12"/>
+      <c r="S25" s="12"/>
+      <c r="T25" s="12"/>
+      <c r="U25" s="12"/>
+      <c r="V25" s="12"/>
+    </row>
+    <row r="26" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A26" s="17"/>
       <c r="B26" s="17"/>
       <c r="C26" s="17"/>
@@ -10773,8 +10746,15 @@
       <c r="L26" s="17"/>
       <c r="M26" s="17"/>
       <c r="N26" s="17"/>
-    </row>
-    <row r="27" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="O26" s="9"/>
+      <c r="Q26" s="12"/>
+      <c r="R26" s="12"/>
+      <c r="S26" s="12"/>
+      <c r="T26" s="12"/>
+      <c r="U26" s="12"/>
+      <c r="V26" s="12"/>
+    </row>
+    <row r="27" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A27" s="17"/>
       <c r="B27" s="17"/>
       <c r="C27" s="17"/>
@@ -10789,8 +10769,15 @@
       <c r="L27" s="17"/>
       <c r="M27" s="17"/>
       <c r="N27" s="17"/>
-    </row>
-    <row r="28" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="O27" s="9"/>
+      <c r="Q27" s="12"/>
+      <c r="R27" s="12"/>
+      <c r="S27" s="12"/>
+      <c r="T27" s="12"/>
+      <c r="U27" s="12"/>
+      <c r="V27" s="12"/>
+    </row>
+    <row r="28" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A28" s="17"/>
       <c r="B28" s="17"/>
       <c r="C28" s="17"/>
@@ -10805,8 +10792,15 @@
       <c r="L28" s="17"/>
       <c r="M28" s="17"/>
       <c r="N28" s="17"/>
-    </row>
-    <row r="29" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="O28" s="9"/>
+      <c r="Q28" s="12"/>
+      <c r="R28" s="12"/>
+      <c r="S28" s="12"/>
+      <c r="T28" s="12"/>
+      <c r="U28" s="12"/>
+      <c r="V28" s="12"/>
+    </row>
+    <row r="29" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A29" s="17"/>
       <c r="B29" s="17"/>
       <c r="C29" s="17"/>
@@ -10821,8 +10815,15 @@
       <c r="L29" s="17"/>
       <c r="M29" s="17"/>
       <c r="N29" s="17"/>
-    </row>
-    <row r="30" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="O29" s="9"/>
+      <c r="Q29" s="12"/>
+      <c r="R29" s="12"/>
+      <c r="S29" s="12"/>
+      <c r="T29" s="12"/>
+      <c r="U29" s="12"/>
+      <c r="V29" s="12"/>
+    </row>
+    <row r="30" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A30" s="17"/>
       <c r="B30" s="17"/>
       <c r="C30" s="17"/>
@@ -10837,9 +10838,14 @@
       <c r="L30" s="17"/>
       <c r="M30" s="17"/>
       <c r="N30" s="17"/>
-      <c r="O30" s="9"/>
-    </row>
-    <row r="31" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="Q30" s="12"/>
+      <c r="R30" s="12"/>
+      <c r="S30" s="12"/>
+      <c r="T30" s="12"/>
+      <c r="U30" s="12"/>
+      <c r="V30" s="12"/>
+    </row>
+    <row r="31" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A31" s="17"/>
       <c r="B31" s="17"/>
       <c r="C31" s="17"/>
@@ -10854,15 +10860,14 @@
       <c r="L31" s="17"/>
       <c r="M31" s="17"/>
       <c r="N31" s="17"/>
-      <c r="O31" s="9"/>
-      <c r="Q31" s="12"/>
-      <c r="R31" s="12"/>
-      <c r="S31" s="12"/>
-      <c r="T31" s="12"/>
-      <c r="U31" s="12"/>
-      <c r="V31" s="12"/>
-    </row>
-    <row r="32" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="Q31" s="13"/>
+      <c r="R31" s="16"/>
+      <c r="S31" s="16"/>
+      <c r="T31" s="16"/>
+      <c r="U31" s="16"/>
+      <c r="V31" s="16"/>
+    </row>
+    <row r="32" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A32" s="17"/>
       <c r="B32" s="17"/>
       <c r="C32" s="17"/>
@@ -10877,13 +10882,12 @@
       <c r="L32" s="17"/>
       <c r="M32" s="17"/>
       <c r="N32" s="17"/>
-      <c r="O32" s="9"/>
-      <c r="Q32" s="12"/>
-      <c r="R32" s="12"/>
-      <c r="S32" s="12"/>
-      <c r="T32" s="12"/>
-      <c r="U32" s="12"/>
-      <c r="V32" s="12"/>
+      <c r="Q32" s="14"/>
+      <c r="R32" s="15"/>
+      <c r="S32" s="15"/>
+      <c r="T32" s="15"/>
+      <c r="U32" s="15"/>
+      <c r="V32" s="15"/>
     </row>
     <row r="33" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A33" s="17"/>
@@ -10900,13 +10904,6 @@
       <c r="L33" s="17"/>
       <c r="M33" s="17"/>
       <c r="N33" s="17"/>
-      <c r="O33" s="9"/>
-      <c r="Q33" s="12"/>
-      <c r="R33" s="12"/>
-      <c r="S33" s="12"/>
-      <c r="T33" s="12"/>
-      <c r="U33" s="12"/>
-      <c r="V33" s="12"/>
     </row>
     <row r="34" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A34" s="17"/>
@@ -10923,13 +10920,6 @@
       <c r="L34" s="17"/>
       <c r="M34" s="17"/>
       <c r="N34" s="17"/>
-      <c r="O34" s="9"/>
-      <c r="Q34" s="12"/>
-      <c r="R34" s="12"/>
-      <c r="S34" s="12"/>
-      <c r="T34" s="12"/>
-      <c r="U34" s="12"/>
-      <c r="V34" s="12"/>
     </row>
     <row r="35" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A35" s="17"/>
@@ -10946,13 +10936,6 @@
       <c r="L35" s="17"/>
       <c r="M35" s="17"/>
       <c r="N35" s="17"/>
-      <c r="O35" s="9"/>
-      <c r="Q35" s="12"/>
-      <c r="R35" s="12"/>
-      <c r="S35" s="12"/>
-      <c r="T35" s="12"/>
-      <c r="U35" s="12"/>
-      <c r="V35" s="12"/>
     </row>
     <row r="36" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A36" s="17"/>
@@ -10969,13 +10952,6 @@
       <c r="L36" s="17"/>
       <c r="M36" s="17"/>
       <c r="N36" s="17"/>
-      <c r="O36" s="9"/>
-      <c r="Q36" s="12"/>
-      <c r="R36" s="12"/>
-      <c r="S36" s="12"/>
-      <c r="T36" s="12"/>
-      <c r="U36" s="12"/>
-      <c r="V36" s="12"/>
     </row>
     <row r="37" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A37" s="17"/>
@@ -10992,13 +10968,13 @@
       <c r="L37" s="17"/>
       <c r="M37" s="17"/>
       <c r="N37" s="17"/>
-      <c r="O37" s="9"/>
       <c r="Q37" s="12"/>
       <c r="R37" s="12"/>
       <c r="S37" s="12"/>
       <c r="T37" s="12"/>
       <c r="U37" s="12"/>
       <c r="V37" s="12"/>
+      <c r="W37" s="12"/>
     </row>
     <row r="38" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A38" s="17"/>
@@ -11015,13 +10991,6 @@
       <c r="L38" s="17"/>
       <c r="M38" s="17"/>
       <c r="N38" s="17"/>
-      <c r="O38" s="9"/>
-      <c r="Q38" s="12"/>
-      <c r="R38" s="12"/>
-      <c r="S38" s="12"/>
-      <c r="T38" s="12"/>
-      <c r="U38" s="12"/>
-      <c r="V38" s="12"/>
     </row>
     <row r="39" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A39" s="17"/>
@@ -11038,13 +11007,6 @@
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
       <c r="N39" s="17"/>
-      <c r="O39" s="9"/>
-      <c r="Q39" s="12"/>
-      <c r="R39" s="12"/>
-      <c r="S39" s="12"/>
-      <c r="T39" s="12"/>
-      <c r="U39" s="12"/>
-      <c r="V39" s="12"/>
     </row>
     <row r="40" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A40" s="17"/>
@@ -11061,12 +11023,6 @@
       <c r="L40" s="17"/>
       <c r="M40" s="17"/>
       <c r="N40" s="17"/>
-      <c r="Q40" s="12"/>
-      <c r="R40" s="12"/>
-      <c r="S40" s="12"/>
-      <c r="T40" s="12"/>
-      <c r="U40" s="12"/>
-      <c r="V40" s="12"/>
     </row>
     <row r="41" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A41" s="17"/>
@@ -11083,14 +11039,8 @@
       <c r="L41" s="17"/>
       <c r="M41" s="17"/>
       <c r="N41" s="17"/>
-      <c r="Q41" s="13"/>
-      <c r="R41" s="16"/>
-      <c r="S41" s="16"/>
-      <c r="T41" s="16"/>
-      <c r="U41" s="16"/>
-      <c r="V41" s="16"/>
-    </row>
-    <row r="42" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="17"/>
       <c r="B42" s="17"/>
       <c r="C42" s="17"/>
@@ -11105,12 +11055,6 @@
       <c r="L42" s="17"/>
       <c r="M42" s="17"/>
       <c r="N42" s="17"/>
-      <c r="Q42" s="14"/>
-      <c r="R42" s="15"/>
-      <c r="S42" s="15"/>
-      <c r="T42" s="15"/>
-      <c r="U42" s="15"/>
-      <c r="V42" s="15"/>
     </row>
     <row r="43" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A43" s="17"/>
@@ -11128,7 +11072,7 @@
       <c r="M43" s="17"/>
       <c r="N43" s="17"/>
     </row>
-    <row r="44" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A44" s="17"/>
       <c r="B44" s="17"/>
       <c r="C44" s="17"/>
@@ -11143,8 +11087,15 @@
       <c r="L44" s="17"/>
       <c r="M44" s="17"/>
       <c r="N44" s="17"/>
-    </row>
-    <row r="45" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="Q44" s="12"/>
+      <c r="R44" s="12"/>
+      <c r="S44" s="12"/>
+      <c r="T44" s="12"/>
+      <c r="U44" s="12"/>
+      <c r="V44" s="12"/>
+      <c r="W44" s="12"/>
+    </row>
+    <row r="45" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A45" s="17"/>
       <c r="B45" s="17"/>
       <c r="C45" s="17"/>
@@ -11159,8 +11110,15 @@
       <c r="L45" s="17"/>
       <c r="M45" s="17"/>
       <c r="N45" s="17"/>
-    </row>
-    <row r="46" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="Q45" s="12"/>
+      <c r="R45" s="12"/>
+      <c r="S45" s="12"/>
+      <c r="T45" s="12"/>
+      <c r="U45" s="12"/>
+      <c r="V45" s="12"/>
+      <c r="W45" s="12"/>
+    </row>
+    <row r="46" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A46" s="17"/>
       <c r="B46" s="17"/>
       <c r="C46" s="17"/>
@@ -11175,8 +11133,15 @@
       <c r="L46" s="17"/>
       <c r="M46" s="17"/>
       <c r="N46" s="17"/>
-    </row>
-    <row r="47" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="Q46" s="12"/>
+      <c r="R46" s="12"/>
+      <c r="S46" s="12"/>
+      <c r="T46" s="12"/>
+      <c r="U46" s="12"/>
+      <c r="V46" s="12"/>
+      <c r="W46" s="12"/>
+    </row>
+    <row r="47" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A47" s="17"/>
       <c r="B47" s="17"/>
       <c r="C47" s="17"/>
@@ -11199,7 +11164,7 @@
       <c r="V47" s="12"/>
       <c r="W47" s="12"/>
     </row>
-    <row r="48" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A48" s="17"/>
       <c r="B48" s="17"/>
       <c r="C48" s="17"/>
@@ -11214,8 +11179,15 @@
       <c r="L48" s="17"/>
       <c r="M48" s="17"/>
       <c r="N48" s="17"/>
-    </row>
-    <row r="49" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="Q48" s="12"/>
+      <c r="R48" s="12"/>
+      <c r="S48" s="12"/>
+      <c r="T48" s="12"/>
+      <c r="U48" s="12"/>
+      <c r="V48" s="12"/>
+      <c r="W48" s="12"/>
+    </row>
+    <row r="49" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A49" s="17"/>
       <c r="B49" s="17"/>
       <c r="C49" s="17"/>
@@ -11230,8 +11202,15 @@
       <c r="L49" s="17"/>
       <c r="M49" s="17"/>
       <c r="N49" s="17"/>
-    </row>
-    <row r="50" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="Q49" s="12"/>
+      <c r="R49" s="12"/>
+      <c r="S49" s="12"/>
+      <c r="T49" s="12"/>
+      <c r="U49" s="12"/>
+      <c r="V49" s="12"/>
+      <c r="W49" s="12"/>
+    </row>
+    <row r="50" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A50" s="17"/>
       <c r="B50" s="17"/>
       <c r="C50" s="17"/>
@@ -11246,8 +11225,15 @@
       <c r="L50" s="17"/>
       <c r="M50" s="17"/>
       <c r="N50" s="17"/>
-    </row>
-    <row r="51" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="Q50" s="12"/>
+      <c r="R50" s="12"/>
+      <c r="S50" s="12"/>
+      <c r="T50" s="12"/>
+      <c r="U50" s="12"/>
+      <c r="V50" s="12"/>
+      <c r="W50" s="12"/>
+    </row>
+    <row r="51" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A51" s="17"/>
       <c r="B51" s="17"/>
       <c r="C51" s="17"/>
@@ -11262,8 +11248,15 @@
       <c r="L51" s="17"/>
       <c r="M51" s="17"/>
       <c r="N51" s="17"/>
-    </row>
-    <row r="52" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q51" s="12"/>
+      <c r="R51" s="12"/>
+      <c r="S51" s="12"/>
+      <c r="T51" s="12"/>
+      <c r="U51" s="12"/>
+      <c r="V51" s="12"/>
+      <c r="W51" s="12"/>
+    </row>
+    <row r="52" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A52" s="17"/>
       <c r="B52" s="17"/>
       <c r="C52" s="17"/>
@@ -11278,8 +11271,15 @@
       <c r="L52" s="17"/>
       <c r="M52" s="17"/>
       <c r="N52" s="17"/>
-    </row>
-    <row r="53" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="Q52" s="12"/>
+      <c r="R52" s="12"/>
+      <c r="S52" s="12"/>
+      <c r="T52" s="12"/>
+      <c r="U52" s="12"/>
+      <c r="V52" s="12"/>
+      <c r="W52" s="12"/>
+    </row>
+    <row r="53" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A53" s="17"/>
       <c r="B53" s="17"/>
       <c r="C53" s="17"/>
@@ -11294,8 +11294,15 @@
       <c r="L53" s="17"/>
       <c r="M53" s="17"/>
       <c r="N53" s="17"/>
-    </row>
-    <row r="54" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="Q53" s="12"/>
+      <c r="R53" s="12"/>
+      <c r="S53" s="12"/>
+      <c r="T53" s="12"/>
+      <c r="U53" s="12"/>
+      <c r="V53" s="12"/>
+      <c r="W53" s="12"/>
+    </row>
+    <row r="54" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A54" s="17"/>
       <c r="B54" s="17"/>
       <c r="C54" s="17"/>
@@ -11318,7 +11325,7 @@
       <c r="V54" s="12"/>
       <c r="W54" s="12"/>
     </row>
-    <row r="55" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A55" s="17"/>
       <c r="B55" s="17"/>
       <c r="C55" s="17"/>
@@ -11341,7 +11348,7 @@
       <c r="V55" s="12"/>
       <c r="W55" s="12"/>
     </row>
-    <row r="56" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A56" s="17"/>
       <c r="B56" s="17"/>
       <c r="C56" s="17"/>
@@ -11364,7 +11371,7 @@
       <c r="V56" s="12"/>
       <c r="W56" s="12"/>
     </row>
-    <row r="57" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A57" s="17"/>
       <c r="B57" s="17"/>
       <c r="C57" s="17"/>
@@ -11387,7 +11394,7 @@
       <c r="V57" s="12"/>
       <c r="W57" s="12"/>
     </row>
-    <row r="58" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A58" s="17"/>
       <c r="B58" s="17"/>
       <c r="C58" s="17"/>
@@ -11410,7 +11417,7 @@
       <c r="V58" s="12"/>
       <c r="W58" s="12"/>
     </row>
-    <row r="59" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A59" s="17"/>
       <c r="B59" s="17"/>
       <c r="C59" s="17"/>
@@ -11433,7 +11440,7 @@
       <c r="V59" s="12"/>
       <c r="W59" s="12"/>
     </row>
-    <row r="60" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A60" s="17"/>
       <c r="B60" s="17"/>
       <c r="C60" s="17"/>
@@ -11456,7 +11463,7 @@
       <c r="V60" s="12"/>
       <c r="W60" s="12"/>
     </row>
-    <row r="61" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A61" s="17"/>
       <c r="B61" s="17"/>
       <c r="C61" s="17"/>
@@ -11479,7 +11486,7 @@
       <c r="V61" s="12"/>
       <c r="W61" s="12"/>
     </row>
-    <row r="62" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A62" s="17"/>
       <c r="B62" s="17"/>
       <c r="C62" s="17"/>
@@ -11494,15 +11501,15 @@
       <c r="L62" s="17"/>
       <c r="M62" s="17"/>
       <c r="N62" s="17"/>
-      <c r="Q62" s="12"/>
-      <c r="R62" s="12"/>
-      <c r="S62" s="12"/>
-      <c r="T62" s="12"/>
-      <c r="U62" s="12"/>
-      <c r="V62" s="12"/>
-      <c r="W62" s="12"/>
-    </row>
-    <row r="63" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="Q62" s="16"/>
+      <c r="R62" s="13"/>
+      <c r="S62" s="13"/>
+      <c r="T62" s="13"/>
+      <c r="U62" s="13"/>
+      <c r="V62" s="13"/>
+      <c r="W62" s="13"/>
+    </row>
+    <row r="63" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A63" s="17"/>
       <c r="B63" s="17"/>
       <c r="C63" s="17"/>
@@ -11517,13 +11524,13 @@
       <c r="L63" s="17"/>
       <c r="M63" s="17"/>
       <c r="N63" s="17"/>
-      <c r="Q63" s="12"/>
-      <c r="R63" s="12"/>
-      <c r="S63" s="12"/>
-      <c r="T63" s="12"/>
-      <c r="U63" s="12"/>
-      <c r="V63" s="12"/>
-      <c r="W63" s="12"/>
+      <c r="Q63" s="15"/>
+      <c r="R63" s="14"/>
+      <c r="S63" s="14"/>
+      <c r="T63" s="14"/>
+      <c r="U63" s="14"/>
+      <c r="V63" s="14"/>
+      <c r="W63" s="14"/>
     </row>
     <row r="64" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A64" s="17"/>
@@ -11540,15 +11547,8 @@
       <c r="L64" s="17"/>
       <c r="M64" s="17"/>
       <c r="N64" s="17"/>
-      <c r="Q64" s="12"/>
-      <c r="R64" s="12"/>
-      <c r="S64" s="12"/>
-      <c r="T64" s="12"/>
-      <c r="U64" s="12"/>
-      <c r="V64" s="12"/>
-      <c r="W64" s="12"/>
-    </row>
-    <row r="65" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="65" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A65" s="17"/>
       <c r="B65" s="17"/>
       <c r="C65" s="17"/>
@@ -11563,15 +11563,8 @@
       <c r="L65" s="17"/>
       <c r="M65" s="17"/>
       <c r="N65" s="17"/>
-      <c r="Q65" s="12"/>
-      <c r="R65" s="12"/>
-      <c r="S65" s="12"/>
-      <c r="T65" s="12"/>
-      <c r="U65" s="12"/>
-      <c r="V65" s="12"/>
-      <c r="W65" s="12"/>
-    </row>
-    <row r="66" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="66" spans="1:22" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="17"/>
       <c r="B66" s="17"/>
       <c r="C66" s="17"/>
@@ -11586,15 +11579,8 @@
       <c r="L66" s="17"/>
       <c r="M66" s="17"/>
       <c r="N66" s="17"/>
-      <c r="Q66" s="12"/>
-      <c r="R66" s="12"/>
-      <c r="S66" s="12"/>
-      <c r="T66" s="12"/>
-      <c r="U66" s="12"/>
-      <c r="V66" s="12"/>
-      <c r="W66" s="12"/>
-    </row>
-    <row r="67" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="67" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A67" s="17"/>
       <c r="B67" s="17"/>
       <c r="C67" s="17"/>
@@ -11609,15 +11595,8 @@
       <c r="L67" s="17"/>
       <c r="M67" s="17"/>
       <c r="N67" s="17"/>
-      <c r="Q67" s="12"/>
-      <c r="R67" s="12"/>
-      <c r="S67" s="12"/>
-      <c r="T67" s="12"/>
-      <c r="U67" s="12"/>
-      <c r="V67" s="12"/>
-      <c r="W67" s="12"/>
-    </row>
-    <row r="68" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="68" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A68" s="17"/>
       <c r="B68" s="17"/>
       <c r="C68" s="17"/>
@@ -11632,15 +11611,9 @@
       <c r="L68" s="17"/>
       <c r="M68" s="17"/>
       <c r="N68" s="17"/>
-      <c r="Q68" s="12"/>
-      <c r="R68" s="12"/>
-      <c r="S68" s="12"/>
-      <c r="T68" s="12"/>
-      <c r="U68" s="12"/>
-      <c r="V68" s="12"/>
-      <c r="W68" s="12"/>
-    </row>
-    <row r="69" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="O68" s="9"/>
+    </row>
+    <row r="69" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A69" s="17"/>
       <c r="B69" s="17"/>
       <c r="C69" s="17"/>
@@ -11655,15 +11628,15 @@
       <c r="L69" s="17"/>
       <c r="M69" s="17"/>
       <c r="N69" s="17"/>
+      <c r="O69" s="9"/>
       <c r="Q69" s="12"/>
       <c r="R69" s="12"/>
       <c r="S69" s="12"/>
       <c r="T69" s="12"/>
       <c r="U69" s="12"/>
       <c r="V69" s="12"/>
-      <c r="W69" s="12"/>
-    </row>
-    <row r="70" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="70" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A70" s="17"/>
       <c r="B70" s="17"/>
       <c r="C70" s="17"/>
@@ -11678,15 +11651,15 @@
       <c r="L70" s="17"/>
       <c r="M70" s="17"/>
       <c r="N70" s="17"/>
+      <c r="O70" s="9"/>
       <c r="Q70" s="12"/>
       <c r="R70" s="12"/>
       <c r="S70" s="12"/>
       <c r="T70" s="12"/>
       <c r="U70" s="12"/>
       <c r="V70" s="12"/>
-      <c r="W70" s="12"/>
-    </row>
-    <row r="71" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="71" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A71" s="17"/>
       <c r="B71" s="17"/>
       <c r="C71" s="17"/>
@@ -11701,15 +11674,15 @@
       <c r="L71" s="17"/>
       <c r="M71" s="17"/>
       <c r="N71" s="17"/>
+      <c r="O71" s="9"/>
       <c r="Q71" s="12"/>
       <c r="R71" s="12"/>
       <c r="S71" s="12"/>
       <c r="T71" s="12"/>
       <c r="U71" s="12"/>
       <c r="V71" s="12"/>
-      <c r="W71" s="12"/>
-    </row>
-    <row r="72" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="72" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A72" s="17"/>
       <c r="B72" s="17"/>
       <c r="C72" s="17"/>
@@ -11724,15 +11697,15 @@
       <c r="L72" s="17"/>
       <c r="M72" s="17"/>
       <c r="N72" s="17"/>
-      <c r="Q72" s="16"/>
-      <c r="R72" s="13"/>
-      <c r="S72" s="13"/>
-      <c r="T72" s="13"/>
-      <c r="U72" s="13"/>
-      <c r="V72" s="13"/>
-      <c r="W72" s="13"/>
-    </row>
-    <row r="73" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="O72" s="9"/>
+      <c r="Q72" s="12"/>
+      <c r="R72" s="12"/>
+      <c r="S72" s="12"/>
+      <c r="T72" s="12"/>
+      <c r="U72" s="12"/>
+      <c r="V72" s="12"/>
+    </row>
+    <row r="73" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A73" s="17"/>
       <c r="B73" s="17"/>
       <c r="C73" s="17"/>
@@ -11747,15 +11720,15 @@
       <c r="L73" s="17"/>
       <c r="M73" s="17"/>
       <c r="N73" s="17"/>
-      <c r="Q73" s="15"/>
-      <c r="R73" s="14"/>
-      <c r="S73" s="14"/>
-      <c r="T73" s="14"/>
-      <c r="U73" s="14"/>
-      <c r="V73" s="14"/>
-      <c r="W73" s="14"/>
-    </row>
-    <row r="74" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="O73" s="9"/>
+      <c r="Q73" s="12"/>
+      <c r="R73" s="12"/>
+      <c r="S73" s="12"/>
+      <c r="T73" s="12"/>
+      <c r="U73" s="12"/>
+      <c r="V73" s="12"/>
+    </row>
+    <row r="74" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A74" s="17"/>
       <c r="B74" s="17"/>
       <c r="C74" s="17"/>
@@ -11770,8 +11743,15 @@
       <c r="L74" s="17"/>
       <c r="M74" s="17"/>
       <c r="N74" s="17"/>
-    </row>
-    <row r="75" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="O74" s="9"/>
+      <c r="Q74" s="12"/>
+      <c r="R74" s="12"/>
+      <c r="S74" s="12"/>
+      <c r="T74" s="12"/>
+      <c r="U74" s="12"/>
+      <c r="V74" s="12"/>
+    </row>
+    <row r="75" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A75" s="17"/>
       <c r="B75" s="17"/>
       <c r="C75" s="17"/>
@@ -11786,8 +11766,15 @@
       <c r="L75" s="17"/>
       <c r="M75" s="17"/>
       <c r="N75" s="17"/>
-    </row>
-    <row r="76" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="O75" s="9"/>
+      <c r="Q75" s="12"/>
+      <c r="R75" s="12"/>
+      <c r="S75" s="12"/>
+      <c r="T75" s="12"/>
+      <c r="U75" s="12"/>
+      <c r="V75" s="12"/>
+    </row>
+    <row r="76" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A76" s="17"/>
       <c r="B76" s="17"/>
       <c r="C76" s="17"/>
@@ -11802,8 +11789,15 @@
       <c r="L76" s="17"/>
       <c r="M76" s="17"/>
       <c r="N76" s="17"/>
-    </row>
-    <row r="77" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="O76" s="9"/>
+      <c r="Q76" s="12"/>
+      <c r="R76" s="12"/>
+      <c r="S76" s="12"/>
+      <c r="T76" s="12"/>
+      <c r="U76" s="12"/>
+      <c r="V76" s="12"/>
+    </row>
+    <row r="77" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A77" s="17"/>
       <c r="B77" s="17"/>
       <c r="C77" s="17"/>
@@ -11818,8 +11812,15 @@
       <c r="L77" s="17"/>
       <c r="M77" s="17"/>
       <c r="N77" s="17"/>
-    </row>
-    <row r="78" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="O77" s="9"/>
+      <c r="Q77" s="12"/>
+      <c r="R77" s="12"/>
+      <c r="S77" s="12"/>
+      <c r="T77" s="12"/>
+      <c r="U77" s="12"/>
+      <c r="V77" s="12"/>
+    </row>
+    <row r="78" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A78" s="17"/>
       <c r="B78" s="17"/>
       <c r="C78" s="17"/>
@@ -11834,9 +11835,14 @@
       <c r="L78" s="17"/>
       <c r="M78" s="17"/>
       <c r="N78" s="17"/>
-      <c r="O78" s="9"/>
-    </row>
-    <row r="79" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="Q78" s="12"/>
+      <c r="R78" s="12"/>
+      <c r="S78" s="12"/>
+      <c r="T78" s="12"/>
+      <c r="U78" s="12"/>
+      <c r="V78" s="12"/>
+    </row>
+    <row r="79" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A79" s="17"/>
       <c r="B79" s="17"/>
       <c r="C79" s="17"/>
@@ -11851,15 +11857,14 @@
       <c r="L79" s="17"/>
       <c r="M79" s="17"/>
       <c r="N79" s="17"/>
-      <c r="O79" s="9"/>
-      <c r="Q79" s="12"/>
-      <c r="R79" s="12"/>
-      <c r="S79" s="12"/>
-      <c r="T79" s="12"/>
-      <c r="U79" s="12"/>
-      <c r="V79" s="12"/>
-    </row>
-    <row r="80" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+      <c r="Q79" s="13"/>
+      <c r="R79" s="16"/>
+      <c r="S79" s="16"/>
+      <c r="T79" s="16"/>
+      <c r="U79" s="16"/>
+      <c r="V79" s="16"/>
+    </row>
+    <row r="80" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A80" s="17"/>
       <c r="B80" s="17"/>
       <c r="C80" s="17"/>
@@ -11874,13 +11879,12 @@
       <c r="L80" s="17"/>
       <c r="M80" s="17"/>
       <c r="N80" s="17"/>
-      <c r="O80" s="9"/>
-      <c r="Q80" s="12"/>
-      <c r="R80" s="12"/>
-      <c r="S80" s="12"/>
-      <c r="T80" s="12"/>
-      <c r="U80" s="12"/>
-      <c r="V80" s="12"/>
+      <c r="Q80" s="14"/>
+      <c r="R80" s="15"/>
+      <c r="S80" s="15"/>
+      <c r="T80" s="15"/>
+      <c r="U80" s="15"/>
+      <c r="V80" s="15"/>
     </row>
     <row r="81" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A81" s="17"/>
@@ -11897,13 +11901,6 @@
       <c r="L81" s="17"/>
       <c r="M81" s="17"/>
       <c r="N81" s="17"/>
-      <c r="O81" s="9"/>
-      <c r="Q81" s="12"/>
-      <c r="R81" s="12"/>
-      <c r="S81" s="12"/>
-      <c r="T81" s="12"/>
-      <c r="U81" s="12"/>
-      <c r="V81" s="12"/>
     </row>
     <row r="82" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A82" s="17"/>
@@ -11920,13 +11917,6 @@
       <c r="L82" s="17"/>
       <c r="M82" s="17"/>
       <c r="N82" s="17"/>
-      <c r="O82" s="9"/>
-      <c r="Q82" s="12"/>
-      <c r="R82" s="12"/>
-      <c r="S82" s="12"/>
-      <c r="T82" s="12"/>
-      <c r="U82" s="12"/>
-      <c r="V82" s="12"/>
     </row>
     <row r="83" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A83" s="17"/>
@@ -11943,13 +11933,6 @@
       <c r="L83" s="17"/>
       <c r="M83" s="17"/>
       <c r="N83" s="17"/>
-      <c r="O83" s="9"/>
-      <c r="Q83" s="12"/>
-      <c r="R83" s="12"/>
-      <c r="S83" s="12"/>
-      <c r="T83" s="12"/>
-      <c r="U83" s="12"/>
-      <c r="V83" s="12"/>
     </row>
     <row r="84" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A84" s="17"/>
@@ -11966,13 +11949,6 @@
       <c r="L84" s="17"/>
       <c r="M84" s="17"/>
       <c r="N84" s="17"/>
-      <c r="O84" s="9"/>
-      <c r="Q84" s="12"/>
-      <c r="R84" s="12"/>
-      <c r="S84" s="12"/>
-      <c r="T84" s="12"/>
-      <c r="U84" s="12"/>
-      <c r="V84" s="12"/>
     </row>
     <row r="85" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A85" s="17"/>
@@ -11989,13 +11965,13 @@
       <c r="L85" s="17"/>
       <c r="M85" s="17"/>
       <c r="N85" s="17"/>
-      <c r="O85" s="9"/>
       <c r="Q85" s="12"/>
       <c r="R85" s="12"/>
       <c r="S85" s="12"/>
       <c r="T85" s="12"/>
       <c r="U85" s="12"/>
       <c r="V85" s="12"/>
+      <c r="W85" s="12"/>
     </row>
     <row r="86" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A86" s="17"/>
@@ -12012,205 +11988,166 @@
       <c r="L86" s="17"/>
       <c r="M86" s="17"/>
       <c r="N86" s="17"/>
-      <c r="O86" s="9"/>
-      <c r="Q86" s="12"/>
-      <c r="R86" s="12"/>
-      <c r="S86" s="12"/>
-      <c r="T86" s="12"/>
-      <c r="U86" s="12"/>
-      <c r="V86" s="12"/>
-    </row>
-    <row r="87" spans="1:23" ht="15" x14ac:dyDescent="0.2">
-      <c r="A87" s="17"/>
-      <c r="B87" s="17"/>
-      <c r="C87" s="17"/>
-      <c r="D87" s="17"/>
-      <c r="E87" s="17"/>
-      <c r="F87" s="17"/>
-      <c r="G87" s="17"/>
-      <c r="H87" s="17"/>
-      <c r="I87" s="17"/>
-      <c r="J87" s="17"/>
-      <c r="K87" s="17"/>
-      <c r="L87" s="17"/>
-      <c r="M87" s="17"/>
-      <c r="N87" s="17"/>
-      <c r="O87" s="9"/>
-      <c r="Q87" s="12"/>
-      <c r="R87" s="12"/>
-      <c r="S87" s="12"/>
-      <c r="T87" s="12"/>
-      <c r="U87" s="12"/>
-      <c r="V87" s="12"/>
-    </row>
-    <row r="88" spans="1:23" ht="15" x14ac:dyDescent="0.2">
-      <c r="A88" s="17"/>
-      <c r="B88" s="17"/>
-      <c r="C88" s="17"/>
-      <c r="D88" s="17"/>
-      <c r="E88" s="17"/>
-      <c r="F88" s="17"/>
-      <c r="G88" s="17"/>
-      <c r="H88" s="17"/>
-      <c r="I88" s="17"/>
-      <c r="J88" s="17"/>
-      <c r="K88" s="17"/>
-      <c r="L88" s="17"/>
-      <c r="M88" s="17"/>
-      <c r="N88" s="17"/>
-      <c r="Q88" s="12"/>
-      <c r="R88" s="12"/>
-      <c r="S88" s="12"/>
-      <c r="T88" s="12"/>
-      <c r="U88" s="12"/>
-      <c r="V88" s="12"/>
-    </row>
-    <row r="89" spans="1:23" ht="15" x14ac:dyDescent="0.2">
-      <c r="A89" s="17"/>
-      <c r="B89" s="17"/>
-      <c r="C89" s="17"/>
-      <c r="D89" s="17"/>
-      <c r="E89" s="17"/>
-      <c r="F89" s="17"/>
-      <c r="G89" s="17"/>
-      <c r="H89" s="17"/>
-      <c r="I89" s="17"/>
-      <c r="J89" s="17"/>
-      <c r="K89" s="17"/>
-      <c r="L89" s="17"/>
-      <c r="M89" s="17"/>
-      <c r="N89" s="17"/>
-      <c r="Q89" s="13"/>
-      <c r="R89" s="16"/>
-      <c r="S89" s="16"/>
-      <c r="T89" s="16"/>
-      <c r="U89" s="16"/>
-      <c r="V89" s="16"/>
-    </row>
-    <row r="90" spans="1:23" ht="15" x14ac:dyDescent="0.2">
-      <c r="A90" s="17"/>
-      <c r="B90" s="17"/>
-      <c r="C90" s="17"/>
-      <c r="D90" s="17"/>
-      <c r="E90" s="17"/>
-      <c r="F90" s="17"/>
-      <c r="G90" s="17"/>
-      <c r="H90" s="17"/>
-      <c r="I90" s="17"/>
-      <c r="J90" s="17"/>
-      <c r="K90" s="17"/>
-      <c r="L90" s="17"/>
-      <c r="M90" s="17"/>
-      <c r="N90" s="17"/>
-      <c r="Q90" s="14"/>
-      <c r="R90" s="15"/>
-      <c r="S90" s="15"/>
-      <c r="T90" s="15"/>
-      <c r="U90" s="15"/>
-      <c r="V90" s="15"/>
-    </row>
-    <row r="91" spans="1:23" ht="15" x14ac:dyDescent="0.2">
-      <c r="A91" s="17"/>
-      <c r="B91" s="17"/>
-      <c r="C91" s="17"/>
-      <c r="D91" s="17"/>
-      <c r="E91" s="17"/>
-      <c r="F91" s="17"/>
-      <c r="G91" s="17"/>
-      <c r="H91" s="17"/>
-      <c r="I91" s="17"/>
-      <c r="J91" s="17"/>
-      <c r="K91" s="17"/>
-      <c r="L91" s="17"/>
-      <c r="M91" s="17"/>
-      <c r="N91" s="17"/>
-    </row>
-    <row r="92" spans="1:23" ht="15" x14ac:dyDescent="0.2">
-      <c r="A92" s="17"/>
-      <c r="B92" s="17"/>
-      <c r="C92" s="17"/>
-      <c r="D92" s="17"/>
-      <c r="E92" s="17"/>
-      <c r="F92" s="17"/>
-      <c r="G92" s="17"/>
-      <c r="H92" s="17"/>
-      <c r="I92" s="17"/>
-      <c r="J92" s="17"/>
-      <c r="K92" s="17"/>
-      <c r="L92" s="17"/>
-      <c r="M92" s="17"/>
-      <c r="N92" s="17"/>
-    </row>
-    <row r="93" spans="1:23" ht="15" x14ac:dyDescent="0.2">
-      <c r="A93" s="17"/>
-      <c r="B93" s="17"/>
-      <c r="C93" s="17"/>
-      <c r="D93" s="17"/>
-      <c r="E93" s="17"/>
-      <c r="F93" s="17"/>
-      <c r="G93" s="17"/>
-      <c r="H93" s="17"/>
-      <c r="I93" s="17"/>
-      <c r="J93" s="17"/>
-      <c r="K93" s="17"/>
-      <c r="L93" s="17"/>
-      <c r="M93" s="17"/>
-      <c r="N93" s="17"/>
-    </row>
-    <row r="94" spans="1:23" ht="15" x14ac:dyDescent="0.2">
-      <c r="A94" s="17"/>
-      <c r="B94" s="17"/>
-      <c r="C94" s="17"/>
-      <c r="D94" s="17"/>
-      <c r="E94" s="17"/>
-      <c r="F94" s="17"/>
-      <c r="G94" s="17"/>
-      <c r="H94" s="17"/>
-      <c r="I94" s="17"/>
-      <c r="J94" s="17"/>
-      <c r="K94" s="17"/>
-      <c r="L94" s="17"/>
-      <c r="M94" s="17"/>
-      <c r="N94" s="17"/>
-    </row>
-    <row r="95" spans="1:23" ht="15" x14ac:dyDescent="0.2">
-      <c r="A95" s="17"/>
-      <c r="B95" s="17"/>
-      <c r="C95" s="17"/>
-      <c r="D95" s="17"/>
-      <c r="E95" s="17"/>
-      <c r="F95" s="17"/>
-      <c r="G95" s="17"/>
-      <c r="H95" s="17"/>
-      <c r="I95" s="17"/>
-      <c r="J95" s="17"/>
-      <c r="K95" s="17"/>
-      <c r="L95" s="17"/>
-      <c r="M95" s="17"/>
-      <c r="N95" s="17"/>
-      <c r="Q95" s="12"/>
-      <c r="R95" s="12"/>
-      <c r="S95" s="12"/>
-      <c r="T95" s="12"/>
-      <c r="U95" s="12"/>
-      <c r="V95" s="12"/>
-      <c r="W95" s="12"/>
-    </row>
-    <row r="96" spans="1:23" ht="15" x14ac:dyDescent="0.2">
-      <c r="A96" s="17"/>
-      <c r="B96" s="17"/>
-      <c r="C96" s="17"/>
-      <c r="D96" s="17"/>
-      <c r="E96" s="17"/>
-      <c r="F96" s="17"/>
-      <c r="G96" s="17"/>
-      <c r="H96" s="17"/>
-      <c r="I96" s="17"/>
-      <c r="J96" s="17"/>
-      <c r="K96" s="17"/>
-      <c r="L96" s="17"/>
-      <c r="M96" s="17"/>
-      <c r="N96" s="17"/>
+    </row>
+    <row r="87" spans="1:23" x14ac:dyDescent="0.15">
+      <c r="A87" s="1"/>
+      <c r="B87" s="1"/>
+      <c r="C87" s="1"/>
+      <c r="D87" s="1"/>
+      <c r="E87" s="1"/>
+      <c r="F87" s="1"/>
+      <c r="G87" s="1"/>
+      <c r="H87" s="1"/>
+      <c r="I87" s="1"/>
+      <c r="J87" s="1"/>
+      <c r="K87" s="1"/>
+      <c r="L87" s="1"/>
+      <c r="M87" s="1"/>
+      <c r="N87" s="1"/>
+    </row>
+    <row r="88" spans="1:23" x14ac:dyDescent="0.15">
+      <c r="A88" s="1"/>
+      <c r="B88" s="1"/>
+      <c r="C88" s="1"/>
+      <c r="D88" s="1"/>
+      <c r="E88" s="1"/>
+      <c r="F88" s="1"/>
+      <c r="G88" s="1"/>
+      <c r="H88" s="1"/>
+      <c r="I88" s="1"/>
+      <c r="J88" s="1"/>
+      <c r="K88" s="1"/>
+      <c r="L88" s="1"/>
+      <c r="M88" s="1"/>
+      <c r="N88" s="1"/>
+    </row>
+    <row r="89" spans="1:23" x14ac:dyDescent="0.15">
+      <c r="A89" s="1"/>
+      <c r="B89" s="1"/>
+      <c r="C89" s="1"/>
+      <c r="D89" s="1"/>
+      <c r="E89" s="1"/>
+      <c r="F89" s="1"/>
+      <c r="G89" s="1"/>
+      <c r="H89" s="1"/>
+      <c r="I89" s="1"/>
+      <c r="J89" s="1"/>
+      <c r="K89" s="1"/>
+      <c r="L89" s="1"/>
+      <c r="M89" s="1"/>
+      <c r="N89" s="1"/>
+    </row>
+    <row r="90" spans="1:23" x14ac:dyDescent="0.15">
+      <c r="A90" s="1"/>
+      <c r="B90" s="1"/>
+      <c r="C90" s="1"/>
+      <c r="D90" s="1"/>
+      <c r="E90" s="1"/>
+      <c r="F90" s="1"/>
+      <c r="G90" s="1"/>
+      <c r="H90" s="1"/>
+      <c r="I90" s="1"/>
+      <c r="J90" s="1"/>
+      <c r="K90" s="1"/>
+      <c r="L90" s="1"/>
+      <c r="M90" s="1"/>
+      <c r="N90" s="1"/>
+    </row>
+    <row r="91" spans="1:23" x14ac:dyDescent="0.15">
+      <c r="A91" s="1"/>
+      <c r="B91" s="1"/>
+      <c r="C91" s="1"/>
+      <c r="D91" s="1"/>
+      <c r="E91" s="1"/>
+      <c r="F91" s="1"/>
+      <c r="G91" s="1"/>
+      <c r="H91" s="1"/>
+      <c r="I91" s="1"/>
+      <c r="J91" s="1"/>
+      <c r="K91" s="1"/>
+      <c r="L91" s="1"/>
+      <c r="M91" s="1"/>
+      <c r="N91" s="1"/>
+    </row>
+    <row r="92" spans="1:23" x14ac:dyDescent="0.15">
+      <c r="A92" s="1"/>
+      <c r="B92" s="1"/>
+      <c r="C92" s="1"/>
+      <c r="D92" s="1"/>
+      <c r="E92" s="1"/>
+      <c r="F92" s="1"/>
+      <c r="G92" s="1"/>
+      <c r="H92" s="1"/>
+      <c r="I92" s="1"/>
+      <c r="J92" s="1"/>
+      <c r="K92" s="1"/>
+      <c r="L92" s="1"/>
+      <c r="M92" s="1"/>
+      <c r="N92" s="1"/>
+    </row>
+    <row r="93" spans="1:23" x14ac:dyDescent="0.15">
+      <c r="A93" s="1"/>
+      <c r="B93" s="1"/>
+      <c r="C93" s="1"/>
+      <c r="D93" s="1"/>
+      <c r="E93" s="1"/>
+      <c r="F93" s="1"/>
+      <c r="G93" s="1"/>
+      <c r="H93" s="1"/>
+      <c r="I93" s="1"/>
+      <c r="J93" s="1"/>
+      <c r="K93" s="1"/>
+      <c r="L93" s="1"/>
+      <c r="M93" s="1"/>
+      <c r="N93" s="1"/>
+    </row>
+    <row r="94" spans="1:23" x14ac:dyDescent="0.15">
+      <c r="A94" s="1"/>
+      <c r="B94" s="1"/>
+      <c r="C94" s="1"/>
+      <c r="D94" s="1"/>
+      <c r="E94" s="1"/>
+      <c r="F94" s="1"/>
+      <c r="G94" s="1"/>
+      <c r="H94" s="1"/>
+      <c r="I94" s="1"/>
+      <c r="J94" s="1"/>
+      <c r="K94" s="1"/>
+      <c r="L94" s="1"/>
+      <c r="M94" s="1"/>
+      <c r="N94" s="1"/>
+    </row>
+    <row r="95" spans="1:23" x14ac:dyDescent="0.15">
+      <c r="A95" s="1"/>
+      <c r="B95" s="1"/>
+      <c r="C95" s="1"/>
+      <c r="D95" s="1"/>
+      <c r="E95" s="1"/>
+      <c r="F95" s="1"/>
+      <c r="G95" s="1"/>
+      <c r="H95" s="1"/>
+      <c r="I95" s="1"/>
+      <c r="J95" s="1"/>
+      <c r="K95" s="1"/>
+      <c r="L95" s="1"/>
+      <c r="M95" s="1"/>
+      <c r="N95" s="1"/>
+    </row>
+    <row r="96" spans="1:23" x14ac:dyDescent="0.15">
+      <c r="A96" s="1"/>
+      <c r="B96" s="1"/>
+      <c r="C96" s="1"/>
+      <c r="D96" s="1"/>
+      <c r="E96" s="1"/>
+      <c r="F96" s="1"/>
+      <c r="G96" s="1"/>
+      <c r="H96" s="1"/>
+      <c r="I96" s="1"/>
+      <c r="J96" s="1"/>
+      <c r="K96" s="1"/>
+      <c r="L96" s="1"/>
+      <c r="M96" s="1"/>
+      <c r="N96" s="1"/>
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A97" s="1"/>
@@ -12292,166 +12229,6 @@
       <c r="M101" s="1"/>
       <c r="N101" s="1"/>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A102" s="1"/>
-      <c r="B102" s="1"/>
-      <c r="C102" s="1"/>
-      <c r="D102" s="1"/>
-      <c r="E102" s="1"/>
-      <c r="F102" s="1"/>
-      <c r="G102" s="1"/>
-      <c r="H102" s="1"/>
-      <c r="I102" s="1"/>
-      <c r="J102" s="1"/>
-      <c r="K102" s="1"/>
-      <c r="L102" s="1"/>
-      <c r="M102" s="1"/>
-      <c r="N102" s="1"/>
-    </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A103" s="1"/>
-      <c r="B103" s="1"/>
-      <c r="C103" s="1"/>
-      <c r="D103" s="1"/>
-      <c r="E103" s="1"/>
-      <c r="F103" s="1"/>
-      <c r="G103" s="1"/>
-      <c r="H103" s="1"/>
-      <c r="I103" s="1"/>
-      <c r="J103" s="1"/>
-      <c r="K103" s="1"/>
-      <c r="L103" s="1"/>
-      <c r="M103" s="1"/>
-      <c r="N103" s="1"/>
-    </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A104" s="1"/>
-      <c r="B104" s="1"/>
-      <c r="C104" s="1"/>
-      <c r="D104" s="1"/>
-      <c r="E104" s="1"/>
-      <c r="F104" s="1"/>
-      <c r="G104" s="1"/>
-      <c r="H104" s="1"/>
-      <c r="I104" s="1"/>
-      <c r="J104" s="1"/>
-      <c r="K104" s="1"/>
-      <c r="L104" s="1"/>
-      <c r="M104" s="1"/>
-      <c r="N104" s="1"/>
-    </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A105" s="1"/>
-      <c r="B105" s="1"/>
-      <c r="C105" s="1"/>
-      <c r="D105" s="1"/>
-      <c r="E105" s="1"/>
-      <c r="F105" s="1"/>
-      <c r="G105" s="1"/>
-      <c r="H105" s="1"/>
-      <c r="I105" s="1"/>
-      <c r="J105" s="1"/>
-      <c r="K105" s="1"/>
-      <c r="L105" s="1"/>
-      <c r="M105" s="1"/>
-      <c r="N105" s="1"/>
-    </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A106" s="1"/>
-      <c r="B106" s="1"/>
-      <c r="C106" s="1"/>
-      <c r="D106" s="1"/>
-      <c r="E106" s="1"/>
-      <c r="F106" s="1"/>
-      <c r="G106" s="1"/>
-      <c r="H106" s="1"/>
-      <c r="I106" s="1"/>
-      <c r="J106" s="1"/>
-      <c r="K106" s="1"/>
-      <c r="L106" s="1"/>
-      <c r="M106" s="1"/>
-      <c r="N106" s="1"/>
-    </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A107" s="1"/>
-      <c r="B107" s="1"/>
-      <c r="C107" s="1"/>
-      <c r="D107" s="1"/>
-      <c r="E107" s="1"/>
-      <c r="F107" s="1"/>
-      <c r="G107" s="1"/>
-      <c r="H107" s="1"/>
-      <c r="I107" s="1"/>
-      <c r="J107" s="1"/>
-      <c r="K107" s="1"/>
-      <c r="L107" s="1"/>
-      <c r="M107" s="1"/>
-      <c r="N107" s="1"/>
-    </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A108" s="1"/>
-      <c r="B108" s="1"/>
-      <c r="C108" s="1"/>
-      <c r="D108" s="1"/>
-      <c r="E108" s="1"/>
-      <c r="F108" s="1"/>
-      <c r="G108" s="1"/>
-      <c r="H108" s="1"/>
-      <c r="I108" s="1"/>
-      <c r="J108" s="1"/>
-      <c r="K108" s="1"/>
-      <c r="L108" s="1"/>
-      <c r="M108" s="1"/>
-      <c r="N108" s="1"/>
-    </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A109" s="1"/>
-      <c r="B109" s="1"/>
-      <c r="C109" s="1"/>
-      <c r="D109" s="1"/>
-      <c r="E109" s="1"/>
-      <c r="F109" s="1"/>
-      <c r="G109" s="1"/>
-      <c r="H109" s="1"/>
-      <c r="I109" s="1"/>
-      <c r="J109" s="1"/>
-      <c r="K109" s="1"/>
-      <c r="L109" s="1"/>
-      <c r="M109" s="1"/>
-      <c r="N109" s="1"/>
-    </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A110" s="1"/>
-      <c r="B110" s="1"/>
-      <c r="C110" s="1"/>
-      <c r="D110" s="1"/>
-      <c r="E110" s="1"/>
-      <c r="F110" s="1"/>
-      <c r="G110" s="1"/>
-      <c r="H110" s="1"/>
-      <c r="I110" s="1"/>
-      <c r="J110" s="1"/>
-      <c r="K110" s="1"/>
-      <c r="L110" s="1"/>
-      <c r="M110" s="1"/>
-      <c r="N110" s="1"/>
-    </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A111" s="1"/>
-      <c r="B111" s="1"/>
-      <c r="C111" s="1"/>
-      <c r="D111" s="1"/>
-      <c r="E111" s="1"/>
-      <c r="F111" s="1"/>
-      <c r="G111" s="1"/>
-      <c r="H111" s="1"/>
-      <c r="I111" s="1"/>
-      <c r="J111" s="1"/>
-      <c r="K111" s="1"/>
-      <c r="L111" s="1"/>
-      <c r="M111" s="1"/>
-      <c r="N111" s="1"/>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A1" location="Contenido!A1" display="Contenido" xr:uid="{6106CCAC-85D3-4A58-8C19-CA66F038BC49}"/>

</xml_diff>